<commit_message>
feat: add beta.2 agenda catalogs and toolchain onboarding
</commit_message>
<xml_diff>
--- a/.SYSTEMX/GLOBAL/ACCESS-MATRIX.xlsx
+++ b/.SYSTEMX/GLOBAL/ACCESS-MATRIX.xlsx
@@ -2,8 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access decisions" sheetId="1" r:id="Ra6cb93356b4b44aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agenda options" sheetId="2" r:id="R936536f411ad4997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access decisions" sheetId="1" r:id="R62134a84cbea4719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agenda options" sheetId="2" r:id="R789aa42c8cd6463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings catalog" sheetId="3" r:id="Ra83872f589b74b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision rules" sheetId="4" r:id="R25f5876352c54802"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent 0 roster" sheetId="5" r:id="R0cc513c9e1a14aad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +17,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -59,8 +62,19 @@
       <x:color rgb="FF7F1D1D"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF13273D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF13273D"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -82,8 +96,33 @@
         <x:fgColor rgb="FFFDECEC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F7FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="10">
     <x:border>
       <x:left/>
       <x:right/>
@@ -151,11 +190,40 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFDCE6F0"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFDCE6F0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFDCE6F0"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFDCE6F0"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="97">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -318,6 +386,162 @@
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
         </x:ext>
       </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1139,4 +1363,1912 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="29" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="56" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="54"/>
+      <x:c r="B1" s="54"/>
+      <x:c r="C1" s="54"/>
+      <x:c r="D1" s="54"/>
+      <x:c r="E1" s="54"/>
+      <x:c r="F1" s="54"/>
+      <x:c r="G1" s="54"/>
+      <x:c r="H1" s="54"/>
+      <x:c r="I1" s="54"/>
+      <x:c r="J1" s="54"/>
+    </x:row>
+    <x:row r="2" ht="31" customHeight="1">
+      <x:c r="A2" s="18" t="str">
+        <x:v>Agenda setting definitions</x:v>
+      </x:c>
+      <x:c r="B2" s="54"/>
+      <x:c r="C2" s="54"/>
+      <x:c r="D2" s="54"/>
+      <x:c r="E2" s="54"/>
+      <x:c r="F2" s="54"/>
+      <x:c r="G2" s="54"/>
+      <x:c r="H2" s="54"/>
+      <x:c r="I2" s="54"/>
+      <x:c r="J2" s="54"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="54" t="str">
+        <x:v>Ten fixed settings start unset. A reviewed option is needed to select context; this view does not apply one.</x:v>
+      </x:c>
+      <x:c r="B3" s="54"/>
+      <x:c r="C3" s="54"/>
+      <x:c r="D3" s="54"/>
+      <x:c r="E3" s="54"/>
+      <x:c r="F3" s="54"/>
+      <x:c r="G3" s="54"/>
+      <x:c r="H3" s="54"/>
+      <x:c r="I3" s="54"/>
+      <x:c r="J3" s="54"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="3" t="str">
+        <x:v>Source: .SYSTEMX/AUTOBOT/AGENDA-SETTINGS.json</x:v>
+      </x:c>
+      <x:c r="B4" s="54"/>
+      <x:c r="C4" s="54"/>
+      <x:c r="D4" s="54"/>
+      <x:c r="E4" s="54"/>
+      <x:c r="F4" s="54"/>
+      <x:c r="G4" s="54"/>
+      <x:c r="H4" s="54"/>
+      <x:c r="I4" s="54"/>
+      <x:c r="J4" s="54"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="54"/>
+      <x:c r="B5" s="54"/>
+      <x:c r="C5" s="54"/>
+      <x:c r="D5" s="54"/>
+      <x:c r="E5" s="54"/>
+      <x:c r="F5" s="54"/>
+      <x:c r="G5" s="54"/>
+      <x:c r="H5" s="54"/>
+      <x:c r="I5" s="54"/>
+      <x:c r="J5" s="54"/>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="59" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="B6" s="60" t="str">
+        <x:v>botId</x:v>
+      </x:c>
+      <x:c r="C6" s="60" t="str">
+        <x:v>setting</x:v>
+      </x:c>
+      <x:c r="D6" s="60" t="str">
+        <x:v>defaultValue</x:v>
+      </x:c>
+      <x:c r="E6" s="60" t="str">
+        <x:v>allowedValues</x:v>
+      </x:c>
+      <x:c r="F6" s="60" t="str">
+        <x:v>providerRulesPath</x:v>
+      </x:c>
+      <x:c r="G6" s="60" t="str">
+        <x:v>reviewRequired</x:v>
+      </x:c>
+      <x:c r="H6" s="60" t="str">
+        <x:v>includeRequiresAccessDecision</x:v>
+      </x:c>
+      <x:c r="I6" s="60" t="str">
+        <x:v>reviewQuestion</x:v>
+      </x:c>
+      <x:c r="J6" s="61" t="str">
+        <x:v>effect</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="41" customHeight="1">
+      <x:c r="A7" s="65" t="str">
+        <x:v>SETTING-001</x:v>
+      </x:c>
+      <x:c r="B7" s="65" t="str">
+        <x:v>autobot.design</x:v>
+      </x:c>
+      <x:c r="C7" s="65" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D7" s="71" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E7" s="65" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F7" s="65" t="str">
+        <x:v>AUTOBOT/Design.MD</x:v>
+      </x:c>
+      <x:c r="G7" s="77" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H7" s="77" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I7" s="74" t="str">
+        <x:v>Should Design reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J7" s="74" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="41" customHeight="1">
+      <x:c r="A8" s="67" t="str">
+        <x:v>SETTING-002</x:v>
+      </x:c>
+      <x:c r="B8" s="67" t="str">
+        <x:v>autobot.soul</x:v>
+      </x:c>
+      <x:c r="C8" s="67" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D8" s="72" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E8" s="67" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F8" s="67" t="str">
+        <x:v>AUTOBOT/Soul.MD</x:v>
+      </x:c>
+      <x:c r="G8" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I8" s="75" t="str">
+        <x:v>Should Soul reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J8" s="75" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="41" customHeight="1">
+      <x:c r="A9" s="67" t="str">
+        <x:v>SETTING-003</x:v>
+      </x:c>
+      <x:c r="B9" s="67" t="str">
+        <x:v>autobot.memory</x:v>
+      </x:c>
+      <x:c r="C9" s="67" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D9" s="72" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E9" s="67" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F9" s="67" t="str">
+        <x:v>AUTOBOT/Memory.MD</x:v>
+      </x:c>
+      <x:c r="G9" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H9" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I9" s="75" t="str">
+        <x:v>Should Memory reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J9" s="75" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="41" customHeight="1">
+      <x:c r="A10" s="67" t="str">
+        <x:v>SETTING-004</x:v>
+      </x:c>
+      <x:c r="B10" s="67" t="str">
+        <x:v>autobot.rules</x:v>
+      </x:c>
+      <x:c r="C10" s="67" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D10" s="72" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E10" s="67" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F10" s="67" t="str">
+        <x:v>AUTOBOT/Rules.MD</x:v>
+      </x:c>
+      <x:c r="G10" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H10" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I10" s="75" t="str">
+        <x:v>Should Rules reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J10" s="75" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="41" customHeight="1">
+      <x:c r="A11" s="67" t="str">
+        <x:v>SETTING-005</x:v>
+      </x:c>
+      <x:c r="B11" s="67" t="str">
+        <x:v>autobot.research</x:v>
+      </x:c>
+      <x:c r="C11" s="67" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D11" s="72" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E11" s="67" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F11" s="67" t="str">
+        <x:v>AUTOBOT/Research.MD</x:v>
+      </x:c>
+      <x:c r="G11" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H11" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I11" s="75" t="str">
+        <x:v>Should Research reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J11" s="75" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="41" customHeight="1">
+      <x:c r="A12" s="67" t="str">
+        <x:v>SETTING-006</x:v>
+      </x:c>
+      <x:c r="B12" s="67" t="str">
+        <x:v>autobot.brand</x:v>
+      </x:c>
+      <x:c r="C12" s="67" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D12" s="72" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E12" s="67" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F12" s="67" t="str">
+        <x:v>AUTOBOT/Brand.MD</x:v>
+      </x:c>
+      <x:c r="G12" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H12" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I12" s="75" t="str">
+        <x:v>Should Brand reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J12" s="75" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="41" customHeight="1">
+      <x:c r="A13" s="67" t="str">
+        <x:v>SETTING-007</x:v>
+      </x:c>
+      <x:c r="B13" s="67" t="str">
+        <x:v>autobot.media</x:v>
+      </x:c>
+      <x:c r="C13" s="67" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D13" s="72" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E13" s="67" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F13" s="67" t="str">
+        <x:v>AUTOBOT/Media.MD</x:v>
+      </x:c>
+      <x:c r="G13" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H13" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I13" s="75" t="str">
+        <x:v>Should Media reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J13" s="75" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="41" customHeight="1">
+      <x:c r="A14" s="67" t="str">
+        <x:v>SETTING-008</x:v>
+      </x:c>
+      <x:c r="B14" s="67" t="str">
+        <x:v>autobot.tokens</x:v>
+      </x:c>
+      <x:c r="C14" s="67" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D14" s="72" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E14" s="67" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F14" s="67" t="str">
+        <x:v>AUTOBOT/Tokens.MD</x:v>
+      </x:c>
+      <x:c r="G14" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H14" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I14" s="75" t="str">
+        <x:v>Should Tokens reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J14" s="75" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="41" customHeight="1">
+      <x:c r="A15" s="67" t="str">
+        <x:v>SETTING-009</x:v>
+      </x:c>
+      <x:c r="B15" s="67" t="str">
+        <x:v>autobot.data</x:v>
+      </x:c>
+      <x:c r="C15" s="67" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D15" s="72" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E15" s="67" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F15" s="67" t="str">
+        <x:v>AUTOBOT/Data.MD</x:v>
+      </x:c>
+      <x:c r="G15" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H15" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I15" s="75" t="str">
+        <x:v>Should Data reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J15" s="75" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="41" customHeight="1">
+      <x:c r="A16" s="69" t="str">
+        <x:v>SETTING-010</x:v>
+      </x:c>
+      <x:c r="B16" s="69" t="str">
+        <x:v>autobot.archive</x:v>
+      </x:c>
+      <x:c r="C16" s="69" t="str">
+        <x:v>context_selection</x:v>
+      </x:c>
+      <x:c r="D16" s="73" t="str">
+        <x:v>unset</x:v>
+      </x:c>
+      <x:c r="E16" s="69" t="str">
+        <x:v>include / exclude</x:v>
+      </x:c>
+      <x:c r="F16" s="69" t="str">
+        <x:v>AUTOBOT/Archive.MD</x:v>
+      </x:c>
+      <x:c r="G16" s="79" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H16" s="79" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I16" s="76" t="str">
+        <x:v>Should Archive reference context be included or excluded for this selected scope?</x:v>
+      </x:c>
+      <x:c r="J16" s="76" t="str">
+        <x:v>Advisory context only; no worker, schedule, or permission starts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="54"/>
+      <x:c r="B17" s="54"/>
+      <x:c r="C17" s="54"/>
+      <x:c r="D17" s="54"/>
+      <x:c r="E17" s="54"/>
+      <x:c r="F17" s="54"/>
+      <x:c r="G17" s="54"/>
+      <x:c r="H17" s="54"/>
+      <x:c r="I17" s="54"/>
+      <x:c r="J17" s="54"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="54"/>
+      <x:c r="B18" s="54"/>
+      <x:c r="C18" s="54"/>
+      <x:c r="D18" s="54"/>
+      <x:c r="E18" s="54"/>
+      <x:c r="F18" s="54"/>
+      <x:c r="G18" s="54"/>
+      <x:c r="H18" s="54"/>
+      <x:c r="I18" s="54"/>
+      <x:c r="J18" s="54"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="54"/>
+      <x:c r="B19" s="54"/>
+      <x:c r="C19" s="54"/>
+      <x:c r="D19" s="54"/>
+      <x:c r="E19" s="54"/>
+      <x:c r="F19" s="54"/>
+      <x:c r="G19" s="54"/>
+      <x:c r="H19" s="54"/>
+      <x:c r="I19" s="54"/>
+      <x:c r="J19" s="54"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="54"/>
+      <x:c r="B20" s="54"/>
+      <x:c r="C20" s="54"/>
+      <x:c r="D20" s="54"/>
+      <x:c r="E20" s="54"/>
+      <x:c r="F20" s="54"/>
+      <x:c r="G20" s="54"/>
+      <x:c r="H20" s="54"/>
+      <x:c r="I20" s="54"/>
+      <x:c r="J20" s="54"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="54"/>
+      <x:c r="B21" s="54"/>
+      <x:c r="C21" s="54"/>
+      <x:c r="D21" s="54"/>
+      <x:c r="E21" s="54"/>
+      <x:c r="F21" s="54"/>
+      <x:c r="G21" s="54"/>
+      <x:c r="H21" s="54"/>
+      <x:c r="I21" s="54"/>
+      <x:c r="J21" s="54"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="54"/>
+      <x:c r="B22" s="54"/>
+      <x:c r="C22" s="54"/>
+      <x:c r="D22" s="54"/>
+      <x:c r="E22" s="54"/>
+      <x:c r="F22" s="54"/>
+      <x:c r="G22" s="54"/>
+      <x:c r="H22" s="54"/>
+      <x:c r="I22" s="54"/>
+      <x:c r="J22" s="54"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="54"/>
+      <x:c r="B23" s="54"/>
+      <x:c r="C23" s="54"/>
+      <x:c r="D23" s="54"/>
+      <x:c r="E23" s="54"/>
+      <x:c r="F23" s="54"/>
+      <x:c r="G23" s="54"/>
+      <x:c r="H23" s="54"/>
+      <x:c r="I23" s="54"/>
+      <x:c r="J23" s="54"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="54"/>
+      <x:c r="B24" s="54"/>
+      <x:c r="C24" s="54"/>
+      <x:c r="D24" s="54"/>
+      <x:c r="E24" s="54"/>
+      <x:c r="F24" s="54"/>
+      <x:c r="G24" s="54"/>
+      <x:c r="H24" s="54"/>
+      <x:c r="I24" s="54"/>
+      <x:c r="J24" s="54"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="54"/>
+      <x:c r="B25" s="54"/>
+      <x:c r="C25" s="54"/>
+      <x:c r="D25" s="54"/>
+      <x:c r="E25" s="54"/>
+      <x:c r="F25" s="54"/>
+      <x:c r="G25" s="54"/>
+      <x:c r="H25" s="54"/>
+      <x:c r="I25" s="54"/>
+      <x:c r="J25" s="54"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="54"/>
+      <x:c r="B26" s="54"/>
+      <x:c r="C26" s="54"/>
+      <x:c r="D26" s="54"/>
+      <x:c r="E26" s="54"/>
+      <x:c r="F26" s="54"/>
+      <x:c r="G26" s="54"/>
+      <x:c r="H26" s="54"/>
+      <x:c r="I26" s="54"/>
+      <x:c r="J26" s="54"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="68" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="62" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="29" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="54"/>
+      <x:c r="B1" s="54"/>
+      <x:c r="C1" s="54"/>
+      <x:c r="D1" s="54"/>
+      <x:c r="E1" s="54"/>
+      <x:c r="F1" s="54"/>
+      <x:c r="G1" s="54"/>
+      <x:c r="H1" s="54"/>
+    </x:row>
+    <x:row r="2" ht="31" customHeight="1">
+      <x:c r="A2" s="18" t="str">
+        <x:v>Access decision rules</x:v>
+      </x:c>
+      <x:c r="B2" s="54"/>
+      <x:c r="C2" s="54"/>
+      <x:c r="D2" s="54"/>
+      <x:c r="E2" s="54"/>
+      <x:c r="F2" s="54"/>
+      <x:c r="G2" s="54"/>
+      <x:c r="H2" s="54"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="54" t="str">
+        <x:v>No row means no grant. Recorded outcomes document review; none changes OS or provider access.</x:v>
+      </x:c>
+      <x:c r="B3" s="54"/>
+      <x:c r="C3" s="54"/>
+      <x:c r="D3" s="54"/>
+      <x:c r="E3" s="54"/>
+      <x:c r="F3" s="54"/>
+      <x:c r="G3" s="54"/>
+      <x:c r="H3" s="54"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="3" t="str">
+        <x:v>Source: .SYSTEMX/GLOBAL/ACCESS-DECISION-RULES.json</x:v>
+      </x:c>
+      <x:c r="B4" s="54"/>
+      <x:c r="C4" s="54"/>
+      <x:c r="D4" s="54"/>
+      <x:c r="E4" s="54"/>
+      <x:c r="F4" s="54"/>
+      <x:c r="G4" s="54"/>
+      <x:c r="H4" s="54"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="54"/>
+      <x:c r="B5" s="54"/>
+      <x:c r="C5" s="54"/>
+      <x:c r="D5" s="54"/>
+      <x:c r="E5" s="54"/>
+      <x:c r="F5" s="54"/>
+      <x:c r="G5" s="54"/>
+      <x:c r="H5" s="54"/>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="59" t="str">
+        <x:v>state</x:v>
+      </x:c>
+      <x:c r="B6" s="60" t="str">
+        <x:v>recorded</x:v>
+      </x:c>
+      <x:c r="C6" s="60" t="str">
+        <x:v>meaning</x:v>
+      </x:c>
+      <x:c r="D6" s="60" t="str">
+        <x:v>policyRefRequiredForNewRecord</x:v>
+      </x:c>
+      <x:c r="E6" s="60" t="str">
+        <x:v>ownerRequired</x:v>
+      </x:c>
+      <x:c r="F6" s="60" t="str">
+        <x:v>evidenceRequired</x:v>
+      </x:c>
+      <x:c r="G6" s="60" t="str">
+        <x:v>identityVerifiedByTemplate</x:v>
+      </x:c>
+      <x:c r="H6" s="61" t="str">
+        <x:v>accessGrantedByTemplate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="41" customHeight="1">
+      <x:c r="A7" s="71" t="str">
+        <x:v>no-row</x:v>
+      </x:c>
+      <x:c r="B7" s="66" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="74" t="str">
+        <x:v>No reviewed decision exists; no access is inferred.</x:v>
+      </x:c>
+      <x:c r="D7" s="77" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="77" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="77" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G7" s="77" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="77" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="41" customHeight="1">
+      <x:c r="A8" s="72" t="str">
+        <x:v>gap</x:v>
+      </x:c>
+      <x:c r="B8" s="68" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" s="75" t="str">
+        <x:v>An access question remains open; resolve it before relying on this path.</x:v>
+      </x:c>
+      <x:c r="D8" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F8" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G8" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="41" customHeight="1">
+      <x:c r="A9" s="72" t="str">
+        <x:v>denied</x:v>
+      </x:c>
+      <x:c r="B9" s="68" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="75" t="str">
+        <x:v>A reviewer recorded denial; do not use this access path.</x:v>
+      </x:c>
+      <x:c r="D9" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F9" s="78" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G9" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="41" customHeight="1">
+      <x:c r="A10" s="73" t="str">
+        <x:v>reviewed-intent</x:v>
+      </x:c>
+      <x:c r="B10" s="70" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="76" t="str">
+        <x:v>A reviewer recorded intended access; verify real identity and permission at the external boundary.</x:v>
+      </x:c>
+      <x:c r="D10" s="79" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="79" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F10" s="79" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G10" s="79" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="79" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="54"/>
+      <x:c r="B11" s="54"/>
+      <x:c r="C11" s="54"/>
+      <x:c r="D11" s="54"/>
+      <x:c r="E11" s="54"/>
+      <x:c r="F11" s="54"/>
+      <x:c r="G11" s="54"/>
+      <x:c r="H11" s="54"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="54"/>
+      <x:c r="B12" s="54"/>
+      <x:c r="C12" s="54"/>
+      <x:c r="D12" s="54"/>
+      <x:c r="E12" s="54"/>
+      <x:c r="F12" s="54"/>
+      <x:c r="G12" s="54"/>
+      <x:c r="H12" s="54"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="80" t="str">
+        <x:v>Decision scope</x:v>
+      </x:c>
+      <x:c r="B13" s="54" t="str">
+        <x:v>actor + resource + action + environment</x:v>
+      </x:c>
+      <x:c r="C13" s="54"/>
+      <x:c r="D13" s="54"/>
+      <x:c r="E13" s="54"/>
+      <x:c r="F13" s="54"/>
+      <x:c r="G13" s="54"/>
+      <x:c r="H13" s="54"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="80" t="str">
+        <x:v>New record fields</x:v>
+      </x:c>
+      <x:c r="B14" s="54" t="str">
+        <x:v>id, actor, resource, action, environment, decision, owner, evidence, reviewedAt</x:v>
+      </x:c>
+      <x:c r="C14" s="54"/>
+      <x:c r="D14" s="54"/>
+      <x:c r="E14" s="54"/>
+      <x:c r="F14" s="54"/>
+      <x:c r="G14" s="54"/>
+      <x:c r="H14" s="54"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="80" t="str">
+        <x:v>Template grant</x:v>
+      </x:c>
+      <x:c r="B15" s="54" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="C15" s="54"/>
+      <x:c r="D15" s="54"/>
+      <x:c r="E15" s="54"/>
+      <x:c r="F15" s="54"/>
+      <x:c r="G15" s="54"/>
+      <x:c r="H15" s="54"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="54"/>
+      <x:c r="B16" s="54"/>
+      <x:c r="C16" s="54"/>
+      <x:c r="D16" s="54"/>
+      <x:c r="E16" s="54"/>
+      <x:c r="F16" s="54"/>
+      <x:c r="G16" s="54"/>
+      <x:c r="H16" s="54"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="54"/>
+      <x:c r="B17" s="54"/>
+      <x:c r="C17" s="54"/>
+      <x:c r="D17" s="54"/>
+      <x:c r="E17" s="54"/>
+      <x:c r="F17" s="54"/>
+      <x:c r="G17" s="54"/>
+      <x:c r="H17" s="54"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="54"/>
+      <x:c r="B18" s="54"/>
+      <x:c r="C18" s="54"/>
+      <x:c r="D18" s="54"/>
+      <x:c r="E18" s="54"/>
+      <x:c r="F18" s="54"/>
+      <x:c r="G18" s="54"/>
+      <x:c r="H18" s="54"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="54"/>
+      <x:c r="B19" s="54"/>
+      <x:c r="C19" s="54"/>
+      <x:c r="D19" s="54"/>
+      <x:c r="E19" s="54"/>
+      <x:c r="F19" s="54"/>
+      <x:c r="G19" s="54"/>
+      <x:c r="H19" s="54"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="54"/>
+      <x:c r="B20" s="54"/>
+      <x:c r="C20" s="54"/>
+      <x:c r="D20" s="54"/>
+      <x:c r="E20" s="54"/>
+      <x:c r="F20" s="54"/>
+      <x:c r="G20" s="54"/>
+      <x:c r="H20" s="54"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="39" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="31" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="29" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="54"/>
+      <x:c r="B1" s="54"/>
+      <x:c r="C1" s="54"/>
+      <x:c r="D1" s="54"/>
+      <x:c r="E1" s="54"/>
+      <x:c r="F1" s="54"/>
+      <x:c r="G1" s="54"/>
+      <x:c r="H1" s="54"/>
+      <x:c r="I1" s="54"/>
+      <x:c r="J1" s="54"/>
+      <x:c r="K1" s="54"/>
+      <x:c r="L1" s="54"/>
+      <x:c r="M1" s="54"/>
+    </x:row>
+    <x:row r="2" ht="31" customHeight="1">
+      <x:c r="A2" s="18" t="str">
+        <x:v>Agent 0 actor roster</x:v>
+      </x:c>
+      <x:c r="B2" s="54"/>
+      <x:c r="C2" s="54"/>
+      <x:c r="D2" s="54"/>
+      <x:c r="E2" s="54"/>
+      <x:c r="F2" s="54"/>
+      <x:c r="G2" s="54"/>
+      <x:c r="H2" s="54"/>
+      <x:c r="I2" s="54"/>
+      <x:c r="J2" s="54"/>
+      <x:c r="K2" s="54"/>
+      <x:c r="L2" s="54"/>
+      <x:c r="M2" s="54"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="54" t="str">
+        <x:v>Twenty stock actor roles and selected-scope registration states. No row verifies external rights or grants access.</x:v>
+      </x:c>
+      <x:c r="B3" s="54"/>
+      <x:c r="C3" s="54"/>
+      <x:c r="D3" s="54"/>
+      <x:c r="E3" s="54"/>
+      <x:c r="F3" s="54"/>
+      <x:c r="G3" s="54"/>
+      <x:c r="H3" s="54"/>
+      <x:c r="I3" s="54"/>
+      <x:c r="J3" s="54"/>
+      <x:c r="K3" s="54"/>
+      <x:c r="L3" s="54"/>
+      <x:c r="M3" s="54"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="3" t="str">
+        <x:v>Source: .SYSTEMX ROOT roster, AGENTS/REGISTRY.json, AGENTB/BOTS.json, WORK/TASKS.json, GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="B4" s="54"/>
+      <x:c r="C4" s="54"/>
+      <x:c r="D4" s="54"/>
+      <x:c r="E4" s="54"/>
+      <x:c r="F4" s="54"/>
+      <x:c r="G4" s="54"/>
+      <x:c r="H4" s="54"/>
+      <x:c r="I4" s="54"/>
+      <x:c r="J4" s="54"/>
+      <x:c r="K4" s="54"/>
+      <x:c r="L4" s="54"/>
+      <x:c r="M4" s="54"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="3" t="str">
+        <x:v>Source revision: d5523cd1568be60f55bac1b4aeb3b2251c7cd9a13b981703757a42ead0dcec8c</x:v>
+      </x:c>
+      <x:c r="B5" s="54"/>
+      <x:c r="C5" s="54"/>
+      <x:c r="D5" s="54"/>
+      <x:c r="E5" s="54"/>
+      <x:c r="F5" s="54"/>
+      <x:c r="G5" s="54"/>
+      <x:c r="H5" s="54"/>
+      <x:c r="I5" s="54"/>
+      <x:c r="J5" s="54"/>
+      <x:c r="K5" s="54"/>
+      <x:c r="L5" s="54"/>
+      <x:c r="M5" s="54"/>
+    </x:row>
+    <x:row r="6" ht="36" customHeight="1">
+      <x:c r="A6" s="85" t="str">
+        <x:v>actorId</x:v>
+      </x:c>
+      <x:c r="B6" s="86" t="str">
+        <x:v>kind</x:v>
+      </x:c>
+      <x:c r="C6" s="86" t="str">
+        <x:v>displayName</x:v>
+      </x:c>
+      <x:c r="D6" s="86" t="str">
+        <x:v>registrationState</x:v>
+      </x:c>
+      <x:c r="E6" s="86" t="str">
+        <x:v>sourceRecord</x:v>
+      </x:c>
+      <x:c r="F6" s="86" t="str">
+        <x:v>workspace</x:v>
+      </x:c>
+      <x:c r="G6" s="86" t="str">
+        <x:v>providerAlias</x:v>
+      </x:c>
+      <x:c r="H6" s="86" t="str">
+        <x:v>taskCount</x:v>
+      </x:c>
+      <x:c r="I6" s="86" t="str">
+        <x:v>accessDecisionIds</x:v>
+      </x:c>
+      <x:c r="J6" s="86" t="str">
+        <x:v>reviewedIntentCount</x:v>
+      </x:c>
+      <x:c r="K6" s="86" t="str">
+        <x:v>deniedCount</x:v>
+      </x:c>
+      <x:c r="L6" s="86" t="str">
+        <x:v>gapCount</x:v>
+      </x:c>
+      <x:c r="M6" s="87" t="str">
+        <x:v>externalRightsVerified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="39" customHeight="1">
+      <x:c r="A7" s="88" t="str">
+        <x:v>agent.0</x:v>
+      </x:c>
+      <x:c r="B7" s="65" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="C7" s="65" t="str">
+        <x:v>agent.0</x:v>
+      </x:c>
+      <x:c r="D7" s="91" t="str">
+        <x:v>registered</x:v>
+      </x:c>
+      <x:c r="E7" s="65" t="str">
+        <x:v>AGENTS/REGISTRY.json</x:v>
+      </x:c>
+      <x:c r="F7" s="65" t="str">
+        <x:v>AGENTS/agent.0</x:v>
+      </x:c>
+      <x:c r="G7" s="65" t="str"/>
+      <x:c r="H7" s="94" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="65" t="str"/>
+      <x:c r="J7" s="94" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="94" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L7" s="94" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="77" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="39" customHeight="1">
+      <x:c r="A8" s="89" t="str">
+        <x:v>agent.1</x:v>
+      </x:c>
+      <x:c r="B8" s="67" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="C8" s="67" t="str">
+        <x:v>agent.1</x:v>
+      </x:c>
+      <x:c r="D8" s="92" t="str">
+        <x:v>unregistered</x:v>
+      </x:c>
+      <x:c r="E8" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F8" s="67" t="str">
+        <x:v>AGENTS/agent.1</x:v>
+      </x:c>
+      <x:c r="G8" s="67" t="str"/>
+      <x:c r="H8" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="67" t="str"/>
+      <x:c r="J8" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L8" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M8" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="39" customHeight="1">
+      <x:c r="A9" s="89" t="str">
+        <x:v>agent.a</x:v>
+      </x:c>
+      <x:c r="B9" s="67" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="C9" s="67" t="str">
+        <x:v>agent.a</x:v>
+      </x:c>
+      <x:c r="D9" s="92" t="str">
+        <x:v>unregistered</x:v>
+      </x:c>
+      <x:c r="E9" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F9" s="67" t="str">
+        <x:v>AGENTS/agent.a</x:v>
+      </x:c>
+      <x:c r="G9" s="67" t="str"/>
+      <x:c r="H9" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="67" t="str"/>
+      <x:c r="J9" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K9" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L9" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M9" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="39" customHeight="1">
+      <x:c r="A10" s="89" t="str">
+        <x:v>agent.b</x:v>
+      </x:c>
+      <x:c r="B10" s="67" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="C10" s="67" t="str">
+        <x:v>agent.b</x:v>
+      </x:c>
+      <x:c r="D10" s="92" t="str">
+        <x:v>unregistered</x:v>
+      </x:c>
+      <x:c r="E10" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F10" s="67" t="str">
+        <x:v>AGENTS/agent.b</x:v>
+      </x:c>
+      <x:c r="G10" s="67" t="str"/>
+      <x:c r="H10" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="67" t="str"/>
+      <x:c r="J10" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K10" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L10" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M10" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="39" customHeight="1">
+      <x:c r="A11" s="89" t="str">
+        <x:v>agent.x</x:v>
+      </x:c>
+      <x:c r="B11" s="67" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="C11" s="67" t="str">
+        <x:v>agent.x</x:v>
+      </x:c>
+      <x:c r="D11" s="92" t="str">
+        <x:v>unregistered</x:v>
+      </x:c>
+      <x:c r="E11" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F11" s="67" t="str">
+        <x:v>AGENTS/agent.x</x:v>
+      </x:c>
+      <x:c r="G11" s="67" t="str"/>
+      <x:c r="H11" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" s="67" t="str"/>
+      <x:c r="J11" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K11" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L11" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="39" customHeight="1">
+      <x:c r="A12" s="89" t="str">
+        <x:v>agent.y</x:v>
+      </x:c>
+      <x:c r="B12" s="67" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="C12" s="67" t="str">
+        <x:v>agent.y</x:v>
+      </x:c>
+      <x:c r="D12" s="92" t="str">
+        <x:v>unregistered</x:v>
+      </x:c>
+      <x:c r="E12" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F12" s="67" t="str">
+        <x:v>AGENTS/agent.y</x:v>
+      </x:c>
+      <x:c r="G12" s="67" t="str"/>
+      <x:c r="H12" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="67" t="str"/>
+      <x:c r="J12" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K12" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L12" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="39" customHeight="1">
+      <x:c r="A13" s="89" t="str">
+        <x:v>agent.z</x:v>
+      </x:c>
+      <x:c r="B13" s="67" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="C13" s="67" t="str">
+        <x:v>agent.z</x:v>
+      </x:c>
+      <x:c r="D13" s="92" t="str">
+        <x:v>unregistered</x:v>
+      </x:c>
+      <x:c r="E13" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F13" s="67" t="str">
+        <x:v>AGENTS/agent.z</x:v>
+      </x:c>
+      <x:c r="G13" s="67" t="str"/>
+      <x:c r="H13" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="67" t="str"/>
+      <x:c r="J13" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K13" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L13" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="39" customHeight="1">
+      <x:c r="A14" s="89" t="str">
+        <x:v>agent.numeric-worker</x:v>
+      </x:c>
+      <x:c r="B14" s="67" t="str">
+        <x:v>agent-pattern</x:v>
+      </x:c>
+      <x:c r="C14" s="67" t="str">
+        <x:v>agent.numeric-worker</x:v>
+      </x:c>
+      <x:c r="D14" s="92" t="str">
+        <x:v>pattern-only</x:v>
+      </x:c>
+      <x:c r="E14" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F14" s="67" t="str"/>
+      <x:c r="G14" s="67" t="str"/>
+      <x:c r="H14" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" s="67" t="str"/>
+      <x:c r="J14" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K14" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L14" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M14" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="39" customHeight="1">
+      <x:c r="A15" s="89" t="str">
+        <x:v>native.subagent</x:v>
+      </x:c>
+      <x:c r="B15" s="67" t="str">
+        <x:v>subagent-pattern</x:v>
+      </x:c>
+      <x:c r="C15" s="67" t="str">
+        <x:v>native.subagent</x:v>
+      </x:c>
+      <x:c r="D15" s="92" t="str">
+        <x:v>pattern-only</x:v>
+      </x:c>
+      <x:c r="E15" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F15" s="67" t="str"/>
+      <x:c r="G15" s="67" t="str"/>
+      <x:c r="H15" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" s="67" t="str"/>
+      <x:c r="J15" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K15" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L15" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M15" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="39" customHeight="1">
+      <x:c r="A16" s="89" t="str">
+        <x:v>agentb.instance</x:v>
+      </x:c>
+      <x:c r="B16" s="67" t="str">
+        <x:v>bot-pattern</x:v>
+      </x:c>
+      <x:c r="C16" s="67" t="str">
+        <x:v>agentb.instance</x:v>
+      </x:c>
+      <x:c r="D16" s="92" t="str">
+        <x:v>pattern-only</x:v>
+      </x:c>
+      <x:c r="E16" s="67" t="str">
+        <x:v>GLOBAL/ACCESS-MATRIX.json</x:v>
+      </x:c>
+      <x:c r="F16" s="67" t="str"/>
+      <x:c r="G16" s="67" t="str"/>
+      <x:c r="H16" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="67" t="str"/>
+      <x:c r="J16" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K16" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L16" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M16" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39" customHeight="1">
+      <x:c r="A17" s="89" t="str">
+        <x:v>autobot.design</x:v>
+      </x:c>
+      <x:c r="B17" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C17" s="67" t="str">
+        <x:v>Design</x:v>
+      </x:c>
+      <x:c r="D17" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E17" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F17" s="67" t="str">
+        <x:v>AUTOBOT/Design.MD</x:v>
+      </x:c>
+      <x:c r="G17" s="67" t="str"/>
+      <x:c r="H17" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="67" t="str"/>
+      <x:c r="J17" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K17" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L17" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M17" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="39" customHeight="1">
+      <x:c r="A18" s="89" t="str">
+        <x:v>autobot.soul</x:v>
+      </x:c>
+      <x:c r="B18" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C18" s="67" t="str">
+        <x:v>Soul</x:v>
+      </x:c>
+      <x:c r="D18" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E18" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F18" s="67" t="str">
+        <x:v>AUTOBOT/Soul.MD</x:v>
+      </x:c>
+      <x:c r="G18" s="67" t="str"/>
+      <x:c r="H18" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="67" t="str"/>
+      <x:c r="J18" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K18" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L18" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M18" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="39" customHeight="1">
+      <x:c r="A19" s="89" t="str">
+        <x:v>autobot.memory</x:v>
+      </x:c>
+      <x:c r="B19" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C19" s="67" t="str">
+        <x:v>Memory</x:v>
+      </x:c>
+      <x:c r="D19" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E19" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F19" s="67" t="str">
+        <x:v>AUTOBOT/Memory.MD</x:v>
+      </x:c>
+      <x:c r="G19" s="67" t="str"/>
+      <x:c r="H19" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="67" t="str"/>
+      <x:c r="J19" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K19" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L19" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M19" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="39" customHeight="1">
+      <x:c r="A20" s="89" t="str">
+        <x:v>autobot.rules</x:v>
+      </x:c>
+      <x:c r="B20" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C20" s="67" t="str">
+        <x:v>Rules</x:v>
+      </x:c>
+      <x:c r="D20" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E20" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F20" s="67" t="str">
+        <x:v>AUTOBOT/Rules.MD</x:v>
+      </x:c>
+      <x:c r="G20" s="67" t="str"/>
+      <x:c r="H20" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="67" t="str"/>
+      <x:c r="J20" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K20" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L20" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M20" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="39" customHeight="1">
+      <x:c r="A21" s="89" t="str">
+        <x:v>autobot.research</x:v>
+      </x:c>
+      <x:c r="B21" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C21" s="67" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="D21" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E21" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F21" s="67" t="str">
+        <x:v>AUTOBOT/Research.MD</x:v>
+      </x:c>
+      <x:c r="G21" s="67" t="str"/>
+      <x:c r="H21" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" s="67" t="str"/>
+      <x:c r="J21" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K21" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L21" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M21" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="39" customHeight="1">
+      <x:c r="A22" s="89" t="str">
+        <x:v>autobot.brand</x:v>
+      </x:c>
+      <x:c r="B22" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C22" s="67" t="str">
+        <x:v>Brand</x:v>
+      </x:c>
+      <x:c r="D22" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E22" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F22" s="67" t="str">
+        <x:v>AUTOBOT/Brand.MD</x:v>
+      </x:c>
+      <x:c r="G22" s="67" t="str"/>
+      <x:c r="H22" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" s="67" t="str"/>
+      <x:c r="J22" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K22" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L22" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M22" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="39" customHeight="1">
+      <x:c r="A23" s="89" t="str">
+        <x:v>autobot.media</x:v>
+      </x:c>
+      <x:c r="B23" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C23" s="67" t="str">
+        <x:v>Media</x:v>
+      </x:c>
+      <x:c r="D23" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E23" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F23" s="67" t="str">
+        <x:v>AUTOBOT/Media.MD</x:v>
+      </x:c>
+      <x:c r="G23" s="67" t="str"/>
+      <x:c r="H23" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="67" t="str"/>
+      <x:c r="J23" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K23" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L23" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M23" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="39" customHeight="1">
+      <x:c r="A24" s="89" t="str">
+        <x:v>autobot.tokens</x:v>
+      </x:c>
+      <x:c r="B24" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C24" s="67" t="str">
+        <x:v>Tokens</x:v>
+      </x:c>
+      <x:c r="D24" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E24" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F24" s="67" t="str">
+        <x:v>AUTOBOT/Tokens.MD</x:v>
+      </x:c>
+      <x:c r="G24" s="67" t="str"/>
+      <x:c r="H24" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="67" t="str"/>
+      <x:c r="J24" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K24" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M24" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="39" customHeight="1">
+      <x:c r="A25" s="89" t="str">
+        <x:v>autobot.data</x:v>
+      </x:c>
+      <x:c r="B25" s="67" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C25" s="67" t="str">
+        <x:v>Data</x:v>
+      </x:c>
+      <x:c r="D25" s="92" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E25" s="67" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F25" s="67" t="str">
+        <x:v>AUTOBOT/Data.MD</x:v>
+      </x:c>
+      <x:c r="G25" s="67" t="str"/>
+      <x:c r="H25" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I25" s="67" t="str"/>
+      <x:c r="J25" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K25" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L25" s="95" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M25" s="78" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="39" customHeight="1">
+      <x:c r="A26" s="90" t="str">
+        <x:v>autobot.archive</x:v>
+      </x:c>
+      <x:c r="B26" s="69" t="str">
+        <x:v>autobot</x:v>
+      </x:c>
+      <x:c r="C26" s="69" t="str">
+        <x:v>Archive</x:v>
+      </x:c>
+      <x:c r="D26" s="93" t="str">
+        <x:v>catalog-only</x:v>
+      </x:c>
+      <x:c r="E26" s="69" t="str">
+        <x:v>AUTOBOT/CATALOG.json</x:v>
+      </x:c>
+      <x:c r="F26" s="69" t="str">
+        <x:v>AUTOBOT/Archive.MD</x:v>
+      </x:c>
+      <x:c r="G26" s="69" t="str"/>
+      <x:c r="H26" s="96" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I26" s="69" t="str"/>
+      <x:c r="J26" s="96" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K26" s="96" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" s="96" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M26" s="79" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="54"/>
+      <x:c r="B27" s="54"/>
+      <x:c r="C27" s="54"/>
+      <x:c r="D27" s="54"/>
+      <x:c r="E27" s="54"/>
+      <x:c r="F27" s="54"/>
+      <x:c r="G27" s="54"/>
+      <x:c r="H27" s="54"/>
+      <x:c r="I27" s="54"/>
+      <x:c r="J27" s="54"/>
+      <x:c r="K27" s="54"/>
+      <x:c r="L27" s="54"/>
+      <x:c r="M27" s="54"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="54"/>
+      <x:c r="B28" s="54"/>
+      <x:c r="C28" s="54"/>
+      <x:c r="D28" s="54"/>
+      <x:c r="E28" s="54"/>
+      <x:c r="F28" s="54"/>
+      <x:c r="G28" s="54"/>
+      <x:c r="H28" s="54"/>
+      <x:c r="I28" s="54"/>
+      <x:c r="J28" s="54"/>
+      <x:c r="K28" s="54"/>
+      <x:c r="L28" s="54"/>
+      <x:c r="M28" s="54"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="54"/>
+      <x:c r="B29" s="54"/>
+      <x:c r="C29" s="54"/>
+      <x:c r="D29" s="54"/>
+      <x:c r="E29" s="54"/>
+      <x:c r="F29" s="54"/>
+      <x:c r="G29" s="54"/>
+      <x:c r="H29" s="54"/>
+      <x:c r="I29" s="54"/>
+      <x:c r="J29" s="54"/>
+      <x:c r="K29" s="54"/>
+      <x:c r="L29" s="54"/>
+      <x:c r="M29" s="54"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="54"/>
+      <x:c r="B30" s="54"/>
+      <x:c r="C30" s="54"/>
+      <x:c r="D30" s="54"/>
+      <x:c r="E30" s="54"/>
+      <x:c r="F30" s="54"/>
+      <x:c r="G30" s="54"/>
+      <x:c r="H30" s="54"/>
+      <x:c r="I30" s="54"/>
+      <x:c r="J30" s="54"/>
+      <x:c r="K30" s="54"/>
+      <x:c r="L30" s="54"/>
+      <x:c r="M30" s="54"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="54"/>
+      <x:c r="B31" s="54"/>
+      <x:c r="C31" s="54"/>
+      <x:c r="D31" s="54"/>
+      <x:c r="E31" s="54"/>
+      <x:c r="F31" s="54"/>
+      <x:c r="G31" s="54"/>
+      <x:c r="H31" s="54"/>
+      <x:c r="I31" s="54"/>
+      <x:c r="J31" s="54"/>
+      <x:c r="K31" s="54"/>
+      <x:c r="L31" s="54"/>
+      <x:c r="M31" s="54"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="54"/>
+      <x:c r="B32" s="54"/>
+      <x:c r="C32" s="54"/>
+      <x:c r="D32" s="54"/>
+      <x:c r="E32" s="54"/>
+      <x:c r="F32" s="54"/>
+      <x:c r="G32" s="54"/>
+      <x:c r="H32" s="54"/>
+      <x:c r="I32" s="54"/>
+      <x:c r="J32" s="54"/>
+      <x:c r="K32" s="54"/>
+      <x:c r="L32" s="54"/>
+      <x:c r="M32" s="54"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="54"/>
+      <x:c r="B33" s="54"/>
+      <x:c r="C33" s="54"/>
+      <x:c r="D33" s="54"/>
+      <x:c r="E33" s="54"/>
+      <x:c r="F33" s="54"/>
+      <x:c r="G33" s="54"/>
+      <x:c r="H33" s="54"/>
+      <x:c r="I33" s="54"/>
+      <x:c r="J33" s="54"/>
+      <x:c r="K33" s="54"/>
+      <x:c r="L33" s="54"/>
+      <x:c r="M33" s="54"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="54"/>
+      <x:c r="B34" s="54"/>
+      <x:c r="C34" s="54"/>
+      <x:c r="D34" s="54"/>
+      <x:c r="E34" s="54"/>
+      <x:c r="F34" s="54"/>
+      <x:c r="G34" s="54"/>
+      <x:c r="H34" s="54"/>
+      <x:c r="I34" s="54"/>
+      <x:c r="J34" s="54"/>
+      <x:c r="K34" s="54"/>
+      <x:c r="L34" s="54"/>
+      <x:c r="M34" s="54"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="54"/>
+      <x:c r="B35" s="54"/>
+      <x:c r="C35" s="54"/>
+      <x:c r="D35" s="54"/>
+      <x:c r="E35" s="54"/>
+      <x:c r="F35" s="54"/>
+      <x:c r="G35" s="54"/>
+      <x:c r="H35" s="54"/>
+      <x:c r="I35" s="54"/>
+      <x:c r="J35" s="54"/>
+      <x:c r="K35" s="54"/>
+      <x:c r="L35" s="54"/>
+      <x:c r="M35" s="54"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="54"/>
+      <x:c r="B36" s="54"/>
+      <x:c r="C36" s="54"/>
+      <x:c r="D36" s="54"/>
+      <x:c r="E36" s="54"/>
+      <x:c r="F36" s="54"/>
+      <x:c r="G36" s="54"/>
+      <x:c r="H36" s="54"/>
+      <x:c r="I36" s="54"/>
+      <x:c r="J36" s="54"/>
+      <x:c r="K36" s="54"/>
+      <x:c r="L36" s="54"/>
+      <x:c r="M36" s="54"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>